<commit_message>
data: fix metadata summary merged cells around five corrected county records
</commit_message>
<xml_diff>
--- a/语料库/语料样本总览.xlsx
+++ b/语料库/语料样本总览.xlsx
@@ -4428,11 +4428,15 @@
       <x:c r="B7" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C7" s="3"/>
+      <x:c r="C7" s="3" t="str">
+        <x:v>国家</x:v>
+      </x:c>
       <x:c r="D7" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E7" s="3"/>
+      <x:c r="E7" s="3" t="str">
+        <x:v>无</x:v>
+      </x:c>
       <x:c r="F7" s="5" t="s">
         <x:v>25</x:v>
       </x:c>
@@ -5297,11 +5301,15 @@
       <x:c r="B42" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C42" s="3"/>
+      <x:c r="C42" s="3" t="str">
+        <x:v>省</x:v>
+      </x:c>
       <x:c r="D42" s="2" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="E42" s="3"/>
+      <x:c r="E42" s="3" t="str">
+        <x:v>中华人民共和国</x:v>
+      </x:c>
       <x:c r="F42" s="5" t="s">
         <x:v>86</x:v>
       </x:c>
@@ -6105,11 +6113,15 @@
       <x:c r="B74" s="2" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="C74" s="3"/>
+      <x:c r="C74" s="3" t="str">
+        <x:v>市</x:v>
+      </x:c>
       <x:c r="D74" s="2" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="E74" s="7"/>
+      <x:c r="E74" s="7" t="str">
+        <x:v>山西省</x:v>
+      </x:c>
       <x:c r="F74" s="5" t="s">
         <x:v>139</x:v>
       </x:c>
@@ -6338,7 +6350,9 @@
       <x:c r="B83" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C83" s="3"/>
+      <x:c r="C83" s="3" t="str">
+        <x:v>市</x:v>
+      </x:c>
       <x:c r="D83" s="2" t="s">
         <x:v>156</x:v>
       </x:c>
@@ -7825,11 +7839,15 @@
       <x:c r="B142" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C142" s="3"/>
+      <x:c r="C142" s="3" t="str">
+        <x:v>市</x:v>
+      </x:c>
       <x:c r="D142" s="2" t="s">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="E142" s="7"/>
+      <x:c r="E142" s="7" t="str">
+        <x:v>江西省</x:v>
+      </x:c>
       <x:c r="F142" s="5" t="s">
         <x:v>264</x:v>
       </x:c>
@@ -17334,11 +17352,17 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="C2:C20"/>
-    <x:mergeCell ref="C21:C64"/>
-    <x:mergeCell ref="C65:C222"/>
+    <x:mergeCell ref="C2:C5"/>
+    <x:mergeCell ref="C7:C20"/>
+    <x:mergeCell ref="C21:C40"/>
+    <x:mergeCell ref="C42:C64"/>
+    <x:mergeCell ref="C65:C72"/>
+    <x:mergeCell ref="C74:C81"/>
+    <x:mergeCell ref="C83:C140"/>
+    <x:mergeCell ref="C142:C222"/>
     <x:mergeCell ref="C223:C507"/>
-    <x:mergeCell ref="D2:D20"/>
+    <x:mergeCell ref="D2:D5"/>
+    <x:mergeCell ref="D7:D20"/>
     <x:mergeCell ref="D21:D22"/>
     <x:mergeCell ref="D24:D25"/>
     <x:mergeCell ref="D26:D27"/>
@@ -17356,7 +17380,6 @@
     <x:mergeCell ref="D66:D67"/>
     <x:mergeCell ref="D69:D70"/>
     <x:mergeCell ref="D71:D72"/>
-    <x:mergeCell ref="D73:D74"/>
     <x:mergeCell ref="D83:D84"/>
     <x:mergeCell ref="D90:D91"/>
     <x:mergeCell ref="D96:D97"/>
@@ -17393,11 +17416,13 @@
     <x:mergeCell ref="D468:D469"/>
     <x:mergeCell ref="D476:D477"/>
     <x:mergeCell ref="D492:D493"/>
-    <x:mergeCell ref="E2:E20"/>
-    <x:mergeCell ref="E21:E64"/>
+    <x:mergeCell ref="E2:E5"/>
+    <x:mergeCell ref="E7:E20"/>
+    <x:mergeCell ref="E21:E40"/>
+    <x:mergeCell ref="E42:E64"/>
     <x:mergeCell ref="E65:E72"/>
-    <x:mergeCell ref="E73:E77"/>
-    <x:mergeCell ref="E78:E82"/>
+    <x:mergeCell ref="E74:E77"/>
+    <x:mergeCell ref="E78:E81"/>
     <x:mergeCell ref="E83:E92"/>
     <x:mergeCell ref="E93:E95"/>
     <x:mergeCell ref="E96:E100"/>
@@ -17405,7 +17430,7 @@
     <x:mergeCell ref="E116:E125"/>
     <x:mergeCell ref="E126:E131"/>
     <x:mergeCell ref="E132:E139"/>
-    <x:mergeCell ref="E140:E143"/>
+    <x:mergeCell ref="E142:E143"/>
     <x:mergeCell ref="E144:E150"/>
     <x:mergeCell ref="E151:E157"/>
     <x:mergeCell ref="E158:E161"/>

</xml_diff>